<commit_message>
Improving dot matrix printer emulation. The MPS801 for COMMODORE machines is almost now perfect!
</commit_message>
<xml_diff>
--- a/docs/C64Data/Characters.xlsx
+++ b/docs/C64Data/Characters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspaces\EMULATORS\docs\C64Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4385E794-C7F5-4196-A347-08A1F1D0C3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C95F78-0B06-46EC-BF21-92BFC5F53888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{8BB24F7E-EEEF-4DC4-B445-87969509D3BC}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="23028" windowHeight="12948" xr2:uid="{8BB24F7E-EEEF-4DC4-B445-87969509D3BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5EEE827-51B2-4DED-9A97-394114155FC2}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="8" width="2.578125" customWidth="1"/>
@@ -1243,7 +1243,7 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <f t="shared" ref="I25:I29" si="9">A25*$A$2+B25*$B$2+C25*$C$2+D25*$D$2+E25*$E$2+F25*$F$2+G25*$G$2+H25*$H$2</f>
+        <f t="shared" ref="I25:I33" si="9">A25*$A$2+B25*$B$2+C25*$C$2+D25*$D$2+E25*$E$2+F25*$F$2+G25*$G$2+H25*$H$2</f>
         <v>0</v>
       </c>
       <c r="J25" t="str">
@@ -1353,7 +1353,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="14.7" thickTop="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A29">
         <v>0</v>
       </c>
@@ -1383,8 +1383,612 @@
         <v>0</v>
       </c>
     </row>
+    <row r="30" spans="1:10" s="2" customFormat="1" ht="14.7" thickTop="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" s="2">
+        <v>0</v>
+      </c>
+      <c r="B30" s="2">
+        <v>0</v>
+      </c>
+      <c r="C30" s="2">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+      <c r="J30" s="2" t="str">
+        <f>DEC2HEX(I30)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31">
+        <v>0</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31" s="1">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+      <c r="J31" t="str">
+        <f t="shared" ref="J31:J37" si="10">DEC2HEX(I31)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32">
+        <v>0</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+      <c r="J32" t="str">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33">
+        <v>0</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+      <c r="J33" t="str">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34">
+        <v>0</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <f t="shared" ref="I34:I42" si="11">A34*$A$2+B34*$B$2+C34*$C$2+D34*$D$2+E34*$E$2+F34*$F$2+G34*$G$2+H34*$H$2</f>
+        <v>8</v>
+      </c>
+      <c r="J34" t="str">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35">
+        <v>0</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="11"/>
+        <v>8</v>
+      </c>
+      <c r="J35" t="str">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36">
+        <v>0</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J36" t="str">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" s="3" customFormat="1" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A37" s="3">
+        <v>0</v>
+      </c>
+      <c r="B37" s="3">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3">
+        <v>0</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3">
+        <v>0</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J37" s="3" t="str">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A38">
+        <v>0</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" s="2" customFormat="1" ht="14.7" thickTop="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" s="2">
+        <v>0</v>
+      </c>
+      <c r="B39" s="2">
+        <v>0</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2">
+        <v>0</v>
+      </c>
+      <c r="E39" s="2">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2">
+        <v>0</v>
+      </c>
+      <c r="I39" s="2">
+        <f t="shared" si="11"/>
+        <v>32</v>
+      </c>
+      <c r="J39" s="2" t="str">
+        <f>DEC2HEX(I39)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40">
+        <v>0</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" s="1">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="11"/>
+        <v>84</v>
+      </c>
+      <c r="J40" t="str">
+        <f t="shared" ref="J40:J46" si="12">DEC2HEX(I40)</f>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41">
+        <v>0</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="11"/>
+        <v>84</v>
+      </c>
+      <c r="J41" t="str">
+        <f t="shared" si="12"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42">
+        <v>0</v>
+      </c>
+      <c r="B42">
+        <v>0</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="11"/>
+        <v>60</v>
+      </c>
+      <c r="J42" t="str">
+        <f t="shared" si="12"/>
+        <v>3C</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43">
+        <v>0</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <f t="shared" ref="I43:I47" si="13">A43*$A$2+B43*$B$2+C43*$C$2+D43*$D$2+E43*$E$2+F43*$F$2+G43*$G$2+H43*$H$2</f>
+        <v>64</v>
+      </c>
+      <c r="J43" t="str">
+        <f t="shared" si="12"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44">
+        <v>0</v>
+      </c>
+      <c r="B44">
+        <v>0</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J44" t="str">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45">
+        <v>0</v>
+      </c>
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J45" t="str">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" s="3" customFormat="1" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="3">
+        <v>0</v>
+      </c>
+      <c r="B46" s="3">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0</v>
+      </c>
+      <c r="D46" s="3">
+        <v>0</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0</v>
+      </c>
+      <c r="G46" s="3">
+        <v>0</v>
+      </c>
+      <c r="H46" s="3">
+        <v>0</v>
+      </c>
+      <c r="I46" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="14.7" thickTop="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47">
+        <v>0</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:H29">
+  <conditionalFormatting sqref="A3:H47">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>

</xml_diff>